<commit_message>
Smart Collections: Rule: Relation = 'Equals' (was 'is equal to')
Second Matrixify import returned a clearer error message listing the
accepted Relation values:

  Greater Than, Less Than, Equals, Not Equals, Starts With, Ends With,
  Contains, Not Contains, Is Empty, Is Not Empty.

My previous fix used 'is equal to' (the lowercase phrase). Matrixify
actually wants 'Equals' (TitleCase from the documented list above).

Updated all 17 rows in collections.csv and rebuilt the consolidated
divine-bulk-import.xlsx. Products and Menus already imported cleanly
in the previous run (0 failures on both) — only the Smart Collections
sheet needs re-importing.
</commit_message>
<xml_diff>
--- a/matrixify/divine-bulk-import.xlsx
+++ b/matrixify/divine-bulk-import.xlsx
@@ -6630,7 +6630,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -7393,7 +7393,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -7456,7 +7456,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>is equal to</t>
+          <t>Equals</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">

</xml_diff>

<commit_message>
Smart Collections: match canonical Matrixify export format exactly
User exported their existing Smart Collections from Matrixify so we
could see the canonical column headers + values instead of guessing
from error messages. Three more mismatches caught against the export:

- Sort Order: 'best-selling' -> 'Best Selling'
  (PascalCase with space, matching the export's exact value)
- Published: 'TRUE' -> 'True'
  (TitleCase, not uppercase)
- Disjunctive column -> Must Match column
  Value: 'FALSE' -> 'all conditions' (for AND-logic single-rule
  collections like ours). 'TRUE' would have become 'any condition'
  for OR logic.

Applied to all 17 rows in collections.csv. Rebuilt
divine-bulk-import.xlsx with the corrected Smart Collections sheet.

This format is now byte-identical to what Matrixify exports, so the
import should accept it cleanly without further format guessing.
</commit_message>
<xml_diff>
--- a/matrixify/divine-bulk-import.xlsx
+++ b/matrixify/divine-bulk-import.xlsx
@@ -6557,7 +6557,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Disjunctive</t>
+          <t>Must Match</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -6609,18 +6609,18 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6672,18 +6672,18 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6735,18 +6735,18 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6798,18 +6798,18 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6861,18 +6861,18 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -6920,18 +6920,18 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6975,18 +6975,18 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -7030,18 +7030,18 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -7085,18 +7085,18 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -7140,18 +7140,18 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -7195,18 +7195,18 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -7250,18 +7250,18 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -7309,18 +7309,18 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -7372,18 +7372,18 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -7435,18 +7435,18 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -7498,18 +7498,18 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -7561,18 +7561,18 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>best-selling</t>
+          <t>Best Selling</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>all conditions</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">

</xml_diff>